<commit_message>
Add first 26/27 matches
</commit_message>
<xml_diff>
--- a/comps_ffm.xlsx
+++ b/comps_ffm.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcosmarinm/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcosmarinm/Documents/Random/mfudbalmk/mfudbalmk/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F00BBCF8-6127-8846-A4DD-BCE915A1DC0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4202E71-A229-9D45-9B01-630B348A2ECF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="33280" windowHeight="16520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2216" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2661" uniqueCount="271">
   <si>
     <t>ИД</t>
   </si>
@@ -812,6 +812,33 @@
   </si>
   <si>
     <t>Куп на РМ 24/25</t>
+  </si>
+  <si>
+    <t>Општинска Квалитетна Фудбалска Лига Прилеп 26/27</t>
+  </si>
+  <si>
+    <t>Квалитетна ОФЛ Прилеп 26/27</t>
+  </si>
+  <si>
+    <t>2026/2027</t>
+  </si>
+  <si>
+    <t>КУП на ОФС Неготино  26/27</t>
+  </si>
+  <si>
+    <t>Бараж за Втора МФЛ 26/27</t>
+  </si>
+  <si>
+    <t>КУП НА ОФС ПРИЛЕП</t>
+  </si>
+  <si>
+    <t>Бараж за Прва МФЛ 26/27</t>
+  </si>
+  <si>
+    <t>Прва МФЛ 26/27</t>
+  </si>
+  <si>
+    <t>Втора МФЛ 26/27</t>
   </si>
 </sst>
 </file>
@@ -14939,6 +14966,1833 @@
         <v>85</v>
       </c>
     </row>
+    <row r="89" spans="1:68" ht="28" x14ac:dyDescent="0.15">
+      <c r="A89" s="5">
+        <v>11377606</v>
+      </c>
+      <c r="B89" s="6" t="s">
+        <v>262</v>
+      </c>
+      <c r="C89" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="D89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="E89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="F89" s="5">
+        <v>16</v>
+      </c>
+      <c r="G89" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="H89" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="I89" s="5">
+        <v>48</v>
+      </c>
+      <c r="J89" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="K89" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="L89" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="M89" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="N89" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="O89" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="P89" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="R89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="S89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="T89" s="5">
+        <v>4</v>
+      </c>
+      <c r="U89" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="V89" s="5">
+        <v>16</v>
+      </c>
+      <c r="W89" s="5">
+        <v>99</v>
+      </c>
+      <c r="X89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="Y89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="Z89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AA89" s="5">
+        <v>90</v>
+      </c>
+      <c r="AB89" s="5">
+        <v>15</v>
+      </c>
+      <c r="AC89" s="5">
+        <v>30</v>
+      </c>
+      <c r="AD89" s="5">
+        <v>5</v>
+      </c>
+      <c r="AE89" s="5">
+        <v>11</v>
+      </c>
+      <c r="AF89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AG89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AH89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AI89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AJ89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AK89" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="AL89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AM89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AN89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AO89" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="AP89" s="5">
+        <v>18</v>
+      </c>
+      <c r="AQ89" s="5">
+        <v>3</v>
+      </c>
+      <c r="AR89" s="5">
+        <v>1</v>
+      </c>
+      <c r="AS89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AT89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AU89" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="AV89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AW89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AX89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AY89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AZ89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BA89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BB89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BC89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BD89" s="5">
+        <v>3</v>
+      </c>
+      <c r="BE89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BF89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BG89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BH89" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="BI89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BJ89" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="BK89" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="BL89" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BM89" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="BN89" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="BO89" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="90" spans="1:68" ht="28" x14ac:dyDescent="0.15">
+      <c r="A90" s="5">
+        <v>11377924</v>
+      </c>
+      <c r="B90" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="C90" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="D90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="E90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="F90" s="5">
+        <v>21</v>
+      </c>
+      <c r="G90" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="H90" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="I90" s="5">
+        <v>9694325</v>
+      </c>
+      <c r="J90" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="K90" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="L90" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="M90" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="N90" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="O90" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="P90" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="R90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="S90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="T90" s="5">
+        <v>5</v>
+      </c>
+      <c r="U90" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="V90" s="5">
+        <v>16</v>
+      </c>
+      <c r="W90" s="5">
+        <v>99</v>
+      </c>
+      <c r="X90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="Y90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="Z90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AA90" s="5">
+        <v>90</v>
+      </c>
+      <c r="AB90" s="5">
+        <v>15</v>
+      </c>
+      <c r="AC90" s="5">
+        <v>30</v>
+      </c>
+      <c r="AD90" s="5">
+        <v>5</v>
+      </c>
+      <c r="AE90" s="5">
+        <v>11</v>
+      </c>
+      <c r="AF90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AG90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AH90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AI90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AJ90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AK90" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="AL90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AM90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AN90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AO90" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="AP90" s="5">
+        <v>18</v>
+      </c>
+      <c r="AQ90" s="5">
+        <v>3</v>
+      </c>
+      <c r="AR90" s="5">
+        <v>1</v>
+      </c>
+      <c r="AS90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AT90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AU90" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="AV90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AW90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AX90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AY90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AZ90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BA90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BB90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BC90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BD90" s="5">
+        <v>3</v>
+      </c>
+      <c r="BE90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BF90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BG90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BH90" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="BI90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BJ90" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="BK90" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="BL90" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BM90" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="BN90" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="BO90" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="91" spans="1:68" ht="28" x14ac:dyDescent="0.15">
+      <c r="A91" s="5">
+        <v>11389932</v>
+      </c>
+      <c r="B91" s="6" t="s">
+        <v>262</v>
+      </c>
+      <c r="C91" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="D91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="E91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="F91" s="5">
+        <v>16</v>
+      </c>
+      <c r="G91" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="H91" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="I91" s="5">
+        <v>48</v>
+      </c>
+      <c r="J91" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="K91" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="L91" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="M91" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="N91" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="O91" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="P91" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="R91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="S91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="T91" s="5">
+        <v>2</v>
+      </c>
+      <c r="U91" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="V91" s="5">
+        <v>16</v>
+      </c>
+      <c r="W91" s="5">
+        <v>99</v>
+      </c>
+      <c r="X91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="Y91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="Z91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AA91" s="5">
+        <v>90</v>
+      </c>
+      <c r="AB91" s="5">
+        <v>15</v>
+      </c>
+      <c r="AC91" s="5">
+        <v>30</v>
+      </c>
+      <c r="AD91" s="5">
+        <v>5</v>
+      </c>
+      <c r="AE91" s="5">
+        <v>11</v>
+      </c>
+      <c r="AF91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AG91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AH91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AI91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AJ91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AK91" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="AL91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AM91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AN91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AO91" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="AP91" s="5">
+        <v>18</v>
+      </c>
+      <c r="AQ91" s="5">
+        <v>3</v>
+      </c>
+      <c r="AR91" s="5">
+        <v>1</v>
+      </c>
+      <c r="AS91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AT91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AU91" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="AV91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AW91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AX91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AY91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AZ91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BA91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BB91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BC91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BD91" s="5">
+        <v>3</v>
+      </c>
+      <c r="BE91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BF91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BG91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BH91" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="BI91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BJ91" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="BK91" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="BL91" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BM91" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="BN91" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="BO91" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="92" spans="1:68" ht="28" x14ac:dyDescent="0.15">
+      <c r="A92" s="5">
+        <v>11432179</v>
+      </c>
+      <c r="B92" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C92" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="D92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="E92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="F92" s="5">
+        <v>19</v>
+      </c>
+      <c r="G92" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="H92" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="I92" s="5">
+        <v>55</v>
+      </c>
+      <c r="J92" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="K92" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="L92" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="M92" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="N92" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="O92" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="P92" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q92" s="5">
+        <v>1</v>
+      </c>
+      <c r="R92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="S92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="T92" s="5">
+        <v>10</v>
+      </c>
+      <c r="U92" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="V92" s="5">
+        <v>16</v>
+      </c>
+      <c r="W92" s="5">
+        <v>99</v>
+      </c>
+      <c r="X92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="Y92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="Z92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AA92" s="5">
+        <v>90</v>
+      </c>
+      <c r="AB92" s="5">
+        <v>15</v>
+      </c>
+      <c r="AC92" s="5">
+        <v>0</v>
+      </c>
+      <c r="AD92" s="5">
+        <v>0</v>
+      </c>
+      <c r="AE92" s="5">
+        <v>11</v>
+      </c>
+      <c r="AF92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AG92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AH92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AI92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AJ92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AK92" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="AL92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AM92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AN92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AO92" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="AP92" s="5">
+        <v>18</v>
+      </c>
+      <c r="AQ92" s="5">
+        <v>5</v>
+      </c>
+      <c r="AR92" s="5">
+        <v>1</v>
+      </c>
+      <c r="AS92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AT92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AU92" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="AV92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AW92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AX92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AY92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AZ92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BA92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BB92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BC92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BD92" s="5">
+        <v>3</v>
+      </c>
+      <c r="BE92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BF92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BG92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BH92" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="BI92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BJ92" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="BK92" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="BL92" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BM92" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="BN92" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="BO92" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="93" spans="1:68" ht="28" x14ac:dyDescent="0.15">
+      <c r="A93" s="5">
+        <v>11474446</v>
+      </c>
+      <c r="B93" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="C93" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="D93" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="E93" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="F93" s="5">
+        <v>1</v>
+      </c>
+      <c r="G93" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="H93" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="I93" s="5">
+        <v>30</v>
+      </c>
+      <c r="J93" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="K93" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="L93" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="M93" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="N93" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="O93" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="P93" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q93" s="5">
+        <v>2</v>
+      </c>
+      <c r="R93" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="S93" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="T93" s="5">
+        <v>8</v>
+      </c>
+      <c r="U93" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="V93" s="5">
+        <v>16</v>
+      </c>
+      <c r="W93" s="5">
+        <v>99</v>
+      </c>
+      <c r="X93" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="Y93" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="Z93" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AA93" s="5">
+        <v>90</v>
+      </c>
+      <c r="AB93" s="5">
+        <v>15</v>
+      </c>
+      <c r="AC93" s="5">
+        <v>0</v>
+      </c>
+      <c r="AD93" s="5">
+        <v>0</v>
+      </c>
+      <c r="AE93" s="5">
+        <v>11</v>
+      </c>
+      <c r="AF93" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AG93" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AH93" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AI93" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AJ93" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AK93" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="AL93" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AM93" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AN93" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AO93" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="AP93" s="5">
+        <v>22</v>
+      </c>
+      <c r="AQ93" s="5">
+        <v>5</v>
+      </c>
+      <c r="AR93" s="5">
+        <v>0</v>
+      </c>
+      <c r="AS93" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AT93" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AU93" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="AV93" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AW93" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AX93" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AY93" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AZ93" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BA93" s="5">
+        <v>3</v>
+      </c>
+      <c r="BB93" s="5">
+        <v>21</v>
+      </c>
+      <c r="BC93" s="7">
+        <v>37987</v>
+      </c>
+      <c r="BD93" s="5">
+        <v>3</v>
+      </c>
+      <c r="BE93" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BF93" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BG93" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BH93" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="BI93" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="BJ93" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="BK93" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="BL93" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BM93" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="BN93" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="BO93" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="94" spans="1:68" ht="28" x14ac:dyDescent="0.15">
+      <c r="A94" s="5">
+        <v>11497240</v>
+      </c>
+      <c r="B94" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="C94" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="D94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="E94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="F94" s="5">
+        <v>16</v>
+      </c>
+      <c r="G94" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="H94" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="I94" s="5">
+        <v>48</v>
+      </c>
+      <c r="J94" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="K94" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="L94" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="M94" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="N94" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="O94" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="P94" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="R94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="S94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="T94" s="5">
+        <v>2</v>
+      </c>
+      <c r="U94" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="V94" s="5">
+        <v>16</v>
+      </c>
+      <c r="W94" s="5">
+        <v>99</v>
+      </c>
+      <c r="X94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="Y94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="Z94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AA94" s="5">
+        <v>90</v>
+      </c>
+      <c r="AB94" s="5">
+        <v>15</v>
+      </c>
+      <c r="AC94" s="5">
+        <v>30</v>
+      </c>
+      <c r="AD94" s="5">
+        <v>5</v>
+      </c>
+      <c r="AE94" s="5">
+        <v>11</v>
+      </c>
+      <c r="AF94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AG94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AH94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AI94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AJ94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AK94" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="AL94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AM94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AN94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AO94" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="AP94" s="5">
+        <v>18</v>
+      </c>
+      <c r="AQ94" s="5">
+        <v>3</v>
+      </c>
+      <c r="AR94" s="5">
+        <v>1</v>
+      </c>
+      <c r="AS94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AT94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AU94" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="AV94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AW94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AX94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AY94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AZ94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BA94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BB94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BC94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BD94" s="5">
+        <v>3</v>
+      </c>
+      <c r="BE94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BF94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BG94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BH94" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="BI94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BJ94" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="BK94" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="BL94" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BM94" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="BN94" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="BO94" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="95" spans="1:68" ht="28" x14ac:dyDescent="0.15">
+      <c r="A95" s="5">
+        <v>11497444</v>
+      </c>
+      <c r="B95" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="C95" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="D95" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="E95" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="F95" s="5">
+        <v>1</v>
+      </c>
+      <c r="G95" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="H95" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="I95" s="5">
+        <v>45</v>
+      </c>
+      <c r="J95" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="K95" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="L95" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="M95" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="N95" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="O95" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="P95" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q95" s="5">
+        <v>1</v>
+      </c>
+      <c r="R95" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="S95" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="T95" s="5">
+        <v>4</v>
+      </c>
+      <c r="U95" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="V95" s="5">
+        <v>16</v>
+      </c>
+      <c r="W95" s="5">
+        <v>99</v>
+      </c>
+      <c r="X95" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="Y95" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="Z95" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AA95" s="5">
+        <v>90</v>
+      </c>
+      <c r="AB95" s="5">
+        <v>15</v>
+      </c>
+      <c r="AC95" s="5">
+        <v>30</v>
+      </c>
+      <c r="AD95" s="5">
+        <v>5</v>
+      </c>
+      <c r="AE95" s="5">
+        <v>11</v>
+      </c>
+      <c r="AF95" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AG95" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AH95" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AI95" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AJ95" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AK95" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="AL95" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AM95" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AN95" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AO95" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="AP95" s="5">
+        <v>22</v>
+      </c>
+      <c r="AQ95" s="5">
+        <v>5</v>
+      </c>
+      <c r="AR95" s="5">
+        <v>0</v>
+      </c>
+      <c r="AS95" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AT95" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AU95" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="AV95" s="5">
+        <v>10</v>
+      </c>
+      <c r="AW95" s="5">
+        <v>10</v>
+      </c>
+      <c r="AX95" s="5">
+        <v>10</v>
+      </c>
+      <c r="AY95" s="5">
+        <v>22</v>
+      </c>
+      <c r="AZ95" s="5">
+        <v>1</v>
+      </c>
+      <c r="BA95" s="5">
+        <v>1</v>
+      </c>
+      <c r="BB95" s="5">
+        <v>21</v>
+      </c>
+      <c r="BC95" s="7">
+        <v>37987</v>
+      </c>
+      <c r="BD95" s="5">
+        <v>3</v>
+      </c>
+      <c r="BE95" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BF95" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BG95" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BH95" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="BI95" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="BJ95" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="BK95" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="BL95" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BM95" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="BN95" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="BO95" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="96" spans="1:68" ht="28" x14ac:dyDescent="0.15">
+      <c r="A96" s="5">
+        <v>11902058</v>
+      </c>
+      <c r="B96" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="C96" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="D96" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="E96" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="F96" s="5">
+        <v>1</v>
+      </c>
+      <c r="G96" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="H96" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="I96" s="5">
+        <v>1</v>
+      </c>
+      <c r="J96" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="K96" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="L96" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="M96" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="N96" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="O96" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="P96" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q96" s="5">
+        <v>1</v>
+      </c>
+      <c r="R96" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="S96" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="T96" s="5">
+        <v>10</v>
+      </c>
+      <c r="U96" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="V96" s="5">
+        <v>16</v>
+      </c>
+      <c r="W96" s="5">
+        <v>99</v>
+      </c>
+      <c r="X96" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="Y96" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="Z96" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AA96" s="5">
+        <v>90</v>
+      </c>
+      <c r="AB96" s="5">
+        <v>15</v>
+      </c>
+      <c r="AC96" s="5">
+        <v>30</v>
+      </c>
+      <c r="AD96" s="5">
+        <v>5</v>
+      </c>
+      <c r="AE96" s="5">
+        <v>11</v>
+      </c>
+      <c r="AF96" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AG96" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AH96" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AI96" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AJ96" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AK96" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="AL96" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AM96" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AN96" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AO96" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="AP96" s="5">
+        <v>22</v>
+      </c>
+      <c r="AQ96" s="5">
+        <v>5</v>
+      </c>
+      <c r="AR96" s="5">
+        <v>0</v>
+      </c>
+      <c r="AS96" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AT96" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AU96" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="AV96" s="5">
+        <v>10</v>
+      </c>
+      <c r="AW96" s="5">
+        <v>10</v>
+      </c>
+      <c r="AX96" s="5">
+        <v>10</v>
+      </c>
+      <c r="AY96" s="5">
+        <v>22</v>
+      </c>
+      <c r="AZ96" s="5">
+        <v>1</v>
+      </c>
+      <c r="BA96" s="5">
+        <v>1</v>
+      </c>
+      <c r="BB96" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BC96" s="7">
+        <v>38353</v>
+      </c>
+      <c r="BD96" s="5">
+        <v>3</v>
+      </c>
+      <c r="BE96" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BF96" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BG96" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BH96" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="BI96" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="BJ96" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="BK96" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="BL96" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BM96" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="BN96" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="BO96" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="97" spans="1:67" ht="28" x14ac:dyDescent="0.15">
+      <c r="A97" s="5">
+        <v>11902074</v>
+      </c>
+      <c r="B97" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="C97" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="D97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="E97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="F97" s="5">
+        <v>1</v>
+      </c>
+      <c r="G97" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="H97" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="I97" s="5">
+        <v>2</v>
+      </c>
+      <c r="J97" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="K97" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="L97" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="M97" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="N97" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="O97" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="P97" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q97" s="5">
+        <v>2</v>
+      </c>
+      <c r="R97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="S97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="T97" s="5">
+        <v>14</v>
+      </c>
+      <c r="U97" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="V97" s="5">
+        <v>16</v>
+      </c>
+      <c r="W97" s="5">
+        <v>99</v>
+      </c>
+      <c r="X97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="Y97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="Z97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AA97" s="5">
+        <v>90</v>
+      </c>
+      <c r="AB97" s="5">
+        <v>15</v>
+      </c>
+      <c r="AC97" s="5">
+        <v>30</v>
+      </c>
+      <c r="AD97" s="5">
+        <v>5</v>
+      </c>
+      <c r="AE97" s="5">
+        <v>11</v>
+      </c>
+      <c r="AF97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AG97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AH97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AI97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AJ97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AK97" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="AL97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AM97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AN97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AO97" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="AP97" s="5">
+        <v>18</v>
+      </c>
+      <c r="AQ97" s="5">
+        <v>3</v>
+      </c>
+      <c r="AR97" s="5">
+        <v>1</v>
+      </c>
+      <c r="AS97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AT97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AU97" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="AV97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AW97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AX97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AY97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="AZ97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BA97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BB97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BC97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BD97" s="5">
+        <v>3</v>
+      </c>
+      <c r="BE97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BF97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BG97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BH97" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="BI97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BJ97" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="BK97" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="BL97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BM97" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="BN97" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="BO97" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
     <row r="1048552" ht="13" x14ac:dyDescent="0.15"/>
     <row r="1048553" ht="13" x14ac:dyDescent="0.15"/>
     <row r="1048554" ht="13" x14ac:dyDescent="0.15"/>

</xml_diff>